<commit_message>
dynamic dropdown with json file
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationData.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationData.xlsx
@@ -127,13 +127,19 @@
     <t>PurposeVisit</t>
   </si>
   <si>
-    <t>OCT</t>
+    <t>Review</t>
   </si>
   <si>
     <t>ConsentForm</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Assign doctor</t>
+  </si>
+  <si>
+    <t>Esha</t>
   </si>
   <si>
     <t>PatientSubCategory</t>
@@ -166,7 +172,7 @@
     <t>Patient category</t>
   </si>
   <si>
-    <t>CORPORATE</t>
+    <t>FULL PAYMENT</t>
   </si>
   <si>
     <t>Corporate name</t>
@@ -757,7 +763,7 @@
       <c r="B22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
@@ -766,21 +772,22 @@
       <c r="B23" s="1" t="s">
         <v>42</v>
       </c>
+      <c r="C23" s="2"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="1">
-        <v>50</v>
+      <c r="B24" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="1" t="s">
         <v>45</v>
+      </c>
+      <c r="B25" s="1">
+        <v>50</v>
       </c>
     </row>
     <row r="26">
@@ -798,7 +805,6 @@
       <c r="B27" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C27" s="2"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
@@ -807,6 +813,7 @@
       <c r="B28" s="1" t="s">
         <v>51</v>
       </c>
+      <c r="C28" s="2"/>
     </row>
     <row r="29">
       <c r="A29" t="s">
@@ -855,7 +862,6 @@
       <c r="B34" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="2"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
@@ -864,6 +870,7 @@
       <c r="B35" s="1" t="s">
         <v>65</v>
       </c>
+      <c r="C35" s="2"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
@@ -889,6 +896,14 @@
         <v>71</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Final json commit and new excel commit
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationData.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationData.xlsx
@@ -7,10 +7,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="opRegistrationData" sheetId="1" r:id="rId1"/>
+    <sheet name="DropdownOptions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr/>
 </workbook>
@@ -279,9 +280,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -763,7 +765,6 @@
       <c r="B22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
@@ -773,6 +774,22 @@
         <v>42</v>
       </c>
       <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="3"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
@@ -781,6 +798,22 @@
       <c r="B24" s="1" t="s">
         <v>44</v>
       </c>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24"/>
+      <c r="G24"/>
+      <c r="H24"/>
+      <c r="I24"/>
+      <c r="J24"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="Q24"/>
+      <c r="R24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
@@ -789,6 +822,22 @@
       <c r="B25" s="1">
         <v>50</v>
       </c>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25"/>
+      <c r="F25"/>
+      <c r="G25"/>
+      <c r="H25"/>
+      <c r="I25"/>
+      <c r="J25"/>
+      <c r="K25"/>
+      <c r="L25"/>
+      <c r="M25"/>
+      <c r="N25"/>
+      <c r="O25"/>
+      <c r="P25"/>
+      <c r="Q25"/>
+      <c r="R25"/>
     </row>
     <row r="26">
       <c r="A26" t="s">
@@ -797,6 +846,22 @@
       <c r="B26" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26"/>
+      <c r="F26"/>
+      <c r="G26"/>
+      <c r="H26"/>
+      <c r="I26"/>
+      <c r="J26"/>
+      <c r="K26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+      <c r="N26"/>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
@@ -805,6 +870,22 @@
       <c r="B27" s="1" t="s">
         <v>49</v>
       </c>
+      <c r="C27"/>
+      <c r="D27"/>
+      <c r="E27"/>
+      <c r="F27"/>
+      <c r="G27"/>
+      <c r="H27"/>
+      <c r="I27"/>
+      <c r="J27"/>
+      <c r="K27"/>
+      <c r="L27"/>
+      <c r="M27"/>
+      <c r="N27"/>
+      <c r="O27"/>
+      <c r="P27"/>
+      <c r="Q27"/>
+      <c r="R27"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
@@ -814,6 +895,22 @@
         <v>51</v>
       </c>
       <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
+      <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
+      <c r="S28" s="3"/>
     </row>
     <row r="29">
       <c r="A29" t="s">
@@ -822,6 +919,22 @@
       <c r="B29" s="1" t="s">
         <v>53</v>
       </c>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
+      <c r="F29"/>
+      <c r="G29"/>
+      <c r="H29"/>
+      <c r="I29"/>
+      <c r="J29"/>
+      <c r="K29"/>
+      <c r="L29"/>
+      <c r="M29"/>
+      <c r="N29"/>
+      <c r="O29"/>
+      <c r="P29"/>
+      <c r="Q29"/>
+      <c r="R29"/>
     </row>
     <row r="30">
       <c r="A30" t="s">
@@ -830,6 +943,22 @@
       <c r="B30" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="H30"/>
+      <c r="I30"/>
+      <c r="J30"/>
+      <c r="K30"/>
+      <c r="L30"/>
+      <c r="M30"/>
+      <c r="N30"/>
+      <c r="O30"/>
+      <c r="P30"/>
+      <c r="Q30"/>
+      <c r="R30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
@@ -838,6 +967,22 @@
       <c r="B31" s="1" t="s">
         <v>57</v>
       </c>
+      <c r="C31"/>
+      <c r="D31"/>
+      <c r="E31"/>
+      <c r="F31"/>
+      <c r="G31"/>
+      <c r="H31"/>
+      <c r="I31"/>
+      <c r="J31"/>
+      <c r="K31"/>
+      <c r="L31"/>
+      <c r="M31"/>
+      <c r="N31"/>
+      <c r="O31"/>
+      <c r="P31"/>
+      <c r="Q31"/>
+      <c r="R31"/>
     </row>
     <row r="32">
       <c r="A32" t="s">
@@ -846,6 +991,22 @@
       <c r="B32" s="1" t="s">
         <v>59</v>
       </c>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="E32"/>
+      <c r="F32"/>
+      <c r="G32"/>
+      <c r="H32"/>
+      <c r="I32"/>
+      <c r="J32"/>
+      <c r="K32"/>
+      <c r="L32"/>
+      <c r="M32"/>
+      <c r="N32"/>
+      <c r="O32"/>
+      <c r="P32"/>
+      <c r="Q32"/>
+      <c r="R32"/>
     </row>
     <row r="33">
       <c r="A33" t="s">
@@ -854,6 +1015,22 @@
       <c r="B33" s="1" t="s">
         <v>61</v>
       </c>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
+      <c r="I33"/>
+      <c r="J33"/>
+      <c r="K33"/>
+      <c r="L33"/>
+      <c r="M33"/>
+      <c r="N33"/>
+      <c r="O33"/>
+      <c r="P33"/>
+      <c r="Q33"/>
+      <c r="R33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
@@ -862,6 +1039,22 @@
       <c r="B34" s="1" t="s">
         <v>63</v>
       </c>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="J34"/>
+      <c r="K34"/>
+      <c r="L34"/>
+      <c r="M34"/>
+      <c r="N34"/>
+      <c r="O34"/>
+      <c r="P34"/>
+      <c r="Q34"/>
+      <c r="R34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
@@ -871,6 +1064,22 @@
         <v>65</v>
       </c>
       <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="2"/>
+      <c r="R35" s="2"/>
+      <c r="S35" s="3"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
@@ -906,4 +1115,11 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+</worksheet>
 </file>
</xml_diff>